<commit_message>
progress: 60 village workbooks (sivaramans-llin 2026-10-10T14:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
@@ -458,6 +458,11 @@
           <t>100</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -465,6 +470,11 @@
           <t>101</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -472,6 +482,11 @@
           <t>102</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -479,6 +494,11 @@
           <t>103</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -486,6 +506,11 @@
           <t>104</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17A, 17B, 17C, 18, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -493,6 +518,11 @@
           <t>105</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12A, 13, 14A, 2, 3, 4, 5A, 5B, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -500,6 +530,11 @@
           <t>106</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -507,6 +542,11 @@
           <t>107</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -514,6 +554,11 @@
           <t>108</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2A, 2A2B, 2B, 3, 4, 5A, 5B, 5C, 5D</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -521,6 +566,11 @@
           <t>109</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B1, 2B2, 3, 4A, 4B1, 4B2, 5A1, 5A2, 5B, 6A1A, 6A1B, 6A2, 6A3, 6B1, 6B2, 6C1, 6C2</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -528,6 +578,11 @@
           <t>11</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -535,6 +590,11 @@
           <t>110</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -542,6 +602,11 @@
           <t>111</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -549,6 +614,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -556,6 +626,11 @@
           <t>113</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2B2, 2B3, 2B4, 3, 4, 5, 6A1, 6A2, 6B1, 6B2, 7</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -563,6 +638,11 @@
           <t>114</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -570,6 +650,11 @@
           <t>115</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -577,6 +662,11 @@
           <t>116</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -584,6 +674,11 @@
           <t>117</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -591,6 +686,11 @@
           <t>118</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 2A, 2B, 3A1, 3A2, 3A3, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -598,6 +698,11 @@
           <t>119</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4, 5A, 5B, 6, 7A, 7B1, 7B2</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -605,6 +710,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 3C, 3D, 4A1, 4A2, 4B, 4C, 5, 6, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -612,6 +722,11 @@
           <t>120</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3A, 3B, 3C, 3D, 3E, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -619,6 +734,11 @@
           <t>121</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 12A, 12B, 2A, 2B, 3, 4A, 4B, 5, 6A, 6B, 7A, 7B, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -626,6 +746,11 @@
           <t>122</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 6, 7, 8, 9A, 9B, 9C1, 9C2</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -633,6 +758,11 @@
           <t>123</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -640,6 +770,11 @@
           <t>124</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -647,6 +782,11 @@
           <t>125</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -654,6 +794,11 @@
           <t>126</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -661,6 +806,11 @@
           <t>127</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -668,6 +818,11 @@
           <t>128</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -675,6 +830,11 @@
           <t>129</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B1, 12B2, 13A, 13B, 14, 2, 3A, 3B, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -682,6 +842,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 1A, 1B, 1C, 1D, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -689,6 +854,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -696,6 +866,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A, 3B, 3C, 3D, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -703,6 +878,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2A, 2B, 2C, 3A10, 3A11, 3A12A1, 3A12B, 3A12C, 3A1A1, 3A1A1A1, 3A1A2A, 3A1A2B, 3A1A3, 3A1A4, 3A1A5, 3A1A6, 3A1B, 3A2A, 3A2B, 3A2C, 3A3A1, 3A3B, 3A4, 3A5, 3A6, 3A7, 3A8B, 3A8C, 3A9A1A, 3A9A2, 3A9A3, 3A9B, 3A9C, 3B, 4A1, 4A2A, 4A3A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -710,6 +890,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10A, 11A, 12, 13A, 14A1, 14A2, 15A1, 15A2, 1A, 1B, 1C1, 1C2, 1C3, 1C4, 2A, 2B, 3A, 3B, 4, 5, 6, 7A1, 7A2, 7B, 8, 9A</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -717,6 +902,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3, 4A1, 4A2, 4B, 4C, 5A, 5B, 5C, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -724,6 +914,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -731,6 +926,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A1, 12A2, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -738,6 +938,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 2B, 3B, 4B, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -745,6 +950,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -752,6 +962,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14A, 14B, 15, 16, 1A, 1B, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -759,6 +974,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A10, 3A2, 3A3, 3A4A, 3A4B, 3A5, 3A6, 3A7, 3A8, 3A9, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -766,6 +986,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1, 1A2, 1B, 2, 3B, 6, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -773,6 +998,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -780,6 +1010,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -787,6 +1022,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1, 10B, 11B, 12B, 14B, 15, 16A, 16B, 16C, 16D, 16E, 17, 18, 2B1, 2B2, 2B3, 3, 4, 5, 6B1, 6B2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -794,6 +1034,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15A, 15B, 16, 17A, 17B, 1A, 1B2, 1C, 2B, 3B, 7B, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -801,6 +1046,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 11A, 11B, 11C, 12A, 12B, 12C, 13B, 1A, 1B, 2B, 3B, 4A, 4B, 5A, 5B, 5C1, 5C2, 5C3, 6B, 7B, 8B, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -808,11 +1058,21 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C1, 10C2, 11, 12A, 12B, 13A, 13B, 14, 15, 16, 17, 18A, 18B, 19, 2, 3, 4, 5, 6A, 6B, 7A1, 7A2, 7A3, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
           <t>147</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6, 7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 60 village workbooks (sivaramans-llin 2026-10-10T15:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
@@ -1082,6 +1082,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 13C, 14, 15, 16, 17, 18, 19, 2, 20, 21, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1089,6 +1094,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1, 10A1A, 10B, 10C, 11A, 11B, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 2A, 2B, 3A, 3B, 4, 5A, 5B, 6, 7A, 7B, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1096,6 +1106,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 12, 13A, 13B, 13C, 14A, 14B, 14C, 15, 16A, 16B, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1103,6 +1118,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1110,6 +1130,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1117,6 +1142,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11A, 11B, 12A, 12B, 13A, 13B, 14A, 14B, 14C, 15, 1A, 1B, 2A, 2B, 3A, 3B1, 3B2, 4, 5A, 5B, 5C, 5D, 5E, 6, 7, 8A, 8B1, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1124,6 +1154,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10, 11, 1A2A3A4A5A, 1B, 2B1, 2B2, 3B, 4B, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1131,6 +1166,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A1, 1A2, 1B1, 1B2, 1C1, 1C2, 1D1, 1D2, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1138,6 +1178,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2B, 3A1A1A, 3B, 4, 5B, 6, 7A1, 7A2, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1145,6 +1190,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B11B12B2, 11A, 12A, 12B1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1152,6 +1202,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1159,6 +1214,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3A, 3B, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1166,6 +1226,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2, 3, 4, 5A, 5B1, 5B2, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1173,6 +1238,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4A, 4B1, 4B2, 5, 6, 7A, 7B1, 7B2, 7B3, 7B4, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1180,6 +1250,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1187,6 +1262,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1194,6 +1274,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 7A1, 7A2, 7B, 8A1, 8A2, 8B, 8C, 8D, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1201,6 +1286,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C1, 10C2, 11, 12, 13, 14A, 14B, 14C, 15A1, 15A2, 15B, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 4A1, 4A2, 4B1, 4B2, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1208,6 +1298,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1215,6 +1310,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1222,6 +1322,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1229,6 +1334,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1236,6 +1346,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1243,6 +1358,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>-, 10A, 11A, 12A1, 12A2, 13A, 13B, 14, 2A, 3A, 4, 5, 6A, 6B, 7, 8, 9A</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1250,6 +1370,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A, 3B, 3C, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1257,6 +1382,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14A, 14B, 15A, 15B, 16A1, 16A2, 16B, 17, 18, 19, 2, 3, 4A1, 4A2, 4B, 5, 6A1, 6A2, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1264,6 +1394,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B1, 1B2, 20A, 2A, 2B3B109B20, 3A, 4, 5, 6, 7, 8, 9A</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1271,6 +1406,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1A, 1B1A1A, 1B1A1B, 1B2, 2, 3A1A, 3A1B, 3A2, 3B, 3C, 3D1, 3D2, 4A, 4B, 5A1, 5A2, 5A3, 5A4, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1278,6 +1418,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1285,6 +1430,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A2, 2A3, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1292,6 +1442,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1299,6 +1454,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1306,6 +1466,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B1, 1B2, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1313,6 +1478,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1320,6 +1490,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1327,6 +1502,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A, 3B, 4A, 4B1, 4B2, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1334,6 +1514,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1341,6 +1526,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1348,6 +1538,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2A1, 2A2, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1355,6 +1550,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1362,6 +1562,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1369,6 +1574,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 16, 17, 18, 19, 2A1A, 2A1B, 2A1C, 2A1D, 2A1E, 2A2, 2B1, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 3</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1376,6 +1586,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1383,6 +1598,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1A, 1A1B, 1A2, 1B, 2, 3A1, 3A10, 3A11, 3A12, 3A13, 3A14, 3A2, 3A3, 3A4, 3A5, 3A6, 3A7, 3A8, 3A9, 3B1A, 3B1B, 3B1C, 3B2A, 3B2B1, 3B2B2, 3C, 3D1A1, 3D1B, 3D2, 3E1A1A, 3E1A1B, 3E1A1C, 3E1B, 3E2A1, 3E2B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1390,6 +1610,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10A, 10B, 10C, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 1A1, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1B, 20, 21, 22, 2A1A1, 2A1B, 2A1C, 2A2, 2A3, 2B, 2C, 3A1A, 3A1B, 3A1C, 3A1D, 3A2, 3A3, 3B, 4, 5A1, 5A2, 5A3A, 5A3B, 5A4, 5B, 5C, 5D, 5E, 5F, 5G, 5H, 5I, 6, 6A1A, 6B, 6C, 7, 8, 80, 9</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1397,6 +1622,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 2A1A1, 2B, 3A, 4A1, 4B1A1A1, 4B1B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1404,6 +1634,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1411,6 +1646,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1418,6 +1658,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15A, 15B, 16, 17, 18A, 18B, 19, 1A, 1B1A1A, 1B1B, 1B2A1, 1B2A2, 1B2B, 1B2C, 1B3A, 1B3B, 1B3C, 1C1, 1C2, 20, 21, 2A, 2B1A, 2B1B, 2B2, 2B3, 3A, 3B, 3C, 4A, 4B, 5A1, 5A2, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1425,6 +1670,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18A, 18B, 19A, 19B, 19C, 2, 20, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1432,6 +1682,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1439,6 +1694,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1446,6 +1706,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1453,6 +1718,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8A1, 8A2, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1460,6 +1730,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B1, 14B2, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1467,6 +1742,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 10, 10A1, 10A1B, 10A2, 10B, 10C, 10D1, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A, 2B, 30, 31, 32, 33, 34, 3A1, 3A2, 3B, 4, 5A, 5B, 6A, 6B, 6C, 7A, 7B, 7C, 8A1A, 8B, 9A1, 9A2, 9A3, 9B1A1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1474,6 +1754,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1481,6 +1766,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B1, 1B2, 2, 3, 4, 5, 6A, 6B1, 6B2, 7, 8, 9A, 9B1, 9B2, 9C1, 9C2</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1488,6 +1778,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1495,6 +1790,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1502,6 +1802,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1A, 3A1B, 3A1C, 3A1D, 3A1E, 3A1F, 3A1G, 3A1H, 3A1I, 3A1J, 3A1K, 3A1L, 3A1M, 3A1N, 3A1O, 3A1P, 3A1Q, 3A1R, 3A1S, 3A1T, 3A1U, 3A1V, 3A1W, 3A1X, 3A2A, 3A2B, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1509,6 +1814,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12A, 12B, 13, 14, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1516,6 +1826,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 2A1, 2A2, 2A3, 2B, 2C1, 2C2, 3, 4, 5, 6, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1523,6 +1838,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20A, 20B, 3A, 3B, 3C, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1530,6 +1850,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1537,6 +1862,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B1A, 3B1B, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1544,11 +1874,21 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A1A1, 1A2, 1A3, 1A4, 1B1A, 1B1B, 1B2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1, 2B, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
           <t>40</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 70 village workbooks (sivaramans-llin 2026-10-10T20:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
@@ -1898,6 +1898,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1905,6 +1910,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 4C, 5A1, 5A2, 5B1, 5B2, 5C1A, 5C1B, 5C2, 5D, 5E</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1912,6 +1922,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2A1, 2A2A2, 2A2B1, 2A2B2, 2A2C, 2A2D, 2A3, 2B, 2C, 3, 4A, 4B, 4C, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1919,6 +1934,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13A, 13B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1926,6 +1946,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 11C, 12A1A, 12A1B, 12A2, 12B, 12C, 13, 14, 1A1, 1A2, 1B, 2A, 2B1, 2B2A, 2B2B, 3A, 3B1, 3B2, 4A1, 4A2A, 4A2B, 4B1, 4B2, 4C1, 4C2, 5A, 5B, 5C, 6, 7A, 7B, 8A, 8B, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1933,6 +1958,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1940,6 +1970,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 5C, 5D, 5E, 5F1, 5F2, 5G, 5H, 5I, 5J, 5K, 5L, 5M</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1947,6 +1982,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2, 3, 4, 5A, 5B, 6A, 6B, 7, 8A1, 8A2, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1954,6 +1994,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B, 4C, 4D, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1961,6 +2006,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1968,6 +2018,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 11D, 12, 13A, 13B, 13C, 2A, 2B, 3, 4A, 4B, 5, 6, 7A, 7B, 7C, 7D, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1975,6 +2030,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1982,6 +2042,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1989,6 +2054,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1996,6 +2066,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1A, 1C1B, 1C2, 2A, 2B, 3A, 3B, 3C, 3D, 3E, 3F, 4A1, 4A2, 4B, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2003,6 +2078,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 7E, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2010,6 +2090,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A1, 2A2, 2A3, 2A4A, 2A4B, 2A4C, 2B, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2017,6 +2102,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2024,6 +2114,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2031,6 +2126,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A1, 6A2, 6B, 6C, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2038,6 +2138,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4A, 4B, 4C, 4D, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2045,6 +2150,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2B, 2C, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2052,6 +2162,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2059,6 +2174,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3A, 3B, 4, 5, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2066,6 +2186,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3A, 3B, 4, 5A, 5B, 5C, 6, 7A, 7B, 8A1, 8A2, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2073,6 +2198,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2080,6 +2210,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2087,6 +2222,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 11, 12, 13, 14A, 14B, 14C, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2094,6 +2234,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 14A, 14B, 15, 16, 17, 18, 1A1, 1A2, 1B, 1C, 2A, 2B, 3, 4A, 4B1, 4B2, 4C, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2101,11 +2246,21 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
           <t>69</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4A, 4B, 5, 6A, 6B, 6C, 6D, 6E, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 71 village workbooks (sivaramans-llin 2026-10-10T20:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Annapanaikankuppam_13.36372_80.096592.xlsx
@@ -2270,6 +2270,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 6, 7A, 7B, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2277,6 +2282,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2284,6 +2294,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D1A, 2D1B, 2D2, 3, 4, 5, 6, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2291,6 +2306,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 2, 3, 4, 5A, 5B, 6, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2298,6 +2318,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A1, 13A2, 13A3A, 13A3B, 13B, 13C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2305,6 +2330,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2312,6 +2342,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 14, 1A1, 1A2, 1B, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2319,6 +2354,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13A, 13B, 14, 15, 16, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2326,6 +2366,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2333,6 +2378,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2340,6 +2390,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10B, 11, 12A, 12B, 13A, 13B, 14A, 14B, 15A, 15B1, 15B2A, 15B2B, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2347,6 +2402,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 1D, 2A, 2B, 2C, 2D, 2E1, 2E2, 3, 4, 5, 6A, 6B, 7A, 7B1, 7B2, 8A, 8B1, 8B2, 8C, 9A, 9B, 9C1, 9C2, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2354,6 +2414,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 19C, 19D, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2361,6 +2426,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 12, 13, 14A, 14B, 15, 16, 17, 18, 19, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2368,6 +2438,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2375,6 +2450,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2382,6 +2462,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2389,6 +2474,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 1A, 1B, 2, 3, 4, 5, 6A, 6B, 7, 8, 9A1, 9A2, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2396,6 +2486,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2403,6 +2498,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2410,6 +2510,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2A, 2B, 2C, 3A1, 3A2, 3B, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2417,6 +2522,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2424,6 +2534,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2431,6 +2546,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2438,6 +2558,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2445,6 +2570,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2452,6 +2582,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2459,6 +2594,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2A, 2B, 3A1, 3B, 3C, 4, 5A, 5B, 6, 7A, 7B, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2466,6 +2606,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 2A, 2B, 3A, 3B, 4A, 4B, 4C, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2473,6 +2618,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2480,6 +2630,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2487,11 +2642,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>